<commit_message>
Rename tracker status from In review to In progress
</commit_message>
<xml_diff>
--- a/demo/templates/rtx-spark-campaign-tracker.xlsx
+++ b/demo/templates/rtx-spark-campaign-tracker.xlsx
@@ -72,7 +72,7 @@
     <t>Mike Chen</t>
   </si>
   <si>
-    <t>In review</t>
+    <t>In progress</t>
   </si>
   <si>
     <t>Mike supplied the approved leadership-review package: 2.1× faster time-to-first-token, 38 tokens/second on the fixed 35B workflow, and 22% lower energy per completed workflow.</t>
@@ -1325,7 +1325,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C100">
     <cfRule type="cellIs" dxfId="1" priority="2" stopIfTrue="1" operator="equal">
-      <formula>"In review"</formula>
+      <formula>"In progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C100">
@@ -1350,7 +1350,7 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C100">
     <cfRule type="cellIs" dxfId="1" priority="7" stopIfTrue="1" operator="equal">
-      <formula>"In review"</formula>
+      <formula>"In progress"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7:C100">
@@ -1370,7 +1370,7 @@
   </conditionalFormatting>
   <dataValidations>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="C7:C100">
-      <formula1>"On track,In review,Awaiting update,Blocked,Complete"</formula1>
+      <formula1>"On track,In progress,Awaiting update,Blocked,Complete"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>

</xml_diff>

<commit_message>
Update product specifications, reference tracker, and Second Brain demo content
</commit_message>
<xml_diff>
--- a/demo/templates/rtx-spark-campaign-tracker.xlsx
+++ b/demo/templates/rtx-spark-campaign-tracker.xlsx
@@ -66,7 +66,7 @@
     <t>Notes</t>
   </si>
   <si>
-    <t>Product performance claims</t>
+    <t>Product specifications</t>
   </si>
   <si>
     <t>Mike Chen</t>
@@ -75,10 +75,10 @@
     <t>In progress</t>
   </si>
   <si>
-    <t>Mike supplied the approved leadership-review package: 2.1× faster time-to-first-token, 38 tokens/second on the fixed 35B workflow, and 22% lower energy per completed workflow.</t>
-  </si>
-  <si>
-    <t>Use the figures and required pre-production qualification verbatim; route final external copy through Legal.</t>
+    <t>Mike supplied approved product specifications: Blackwell RTX GPU: Up to 6,144 cores; Grace CPU: Up to 20 cores; FP4 AI performance: Up to 1 petaflop; Unified memory: Up to 128 GB.</t>
+  </si>
+  <si>
+    <t>Keep “up to” with every specification and retain FP4; route final external copy through Legal.</t>
   </si>
   <si>
     <t>Campaign-wide Legal approval remains pending.</t>
@@ -102,7 +102,7 @@
     <t>Slides 4, 7, and 9 now contain the approved leadership-review figures, retail-owner dependency, and shoot-slot options.</t>
   </si>
   <si>
-    <t>Remove slide 6 from the live flow manually and confirm the performance package remains current before presenting.</t>
+    <t>Remove slide 6 from the live flow manually and confirm the specifications package remains current before presenting.</t>
   </si>
   <si>
     <t>Slide 6 still requires manual removal; retail demo owner remains unassigned.</t>
@@ -120,10 +120,10 @@
     <t>Awaiting update</t>
   </si>
   <si>
-    <t>Mike supplied the approved leadership-review figures and required pre-production qualification; Agent Messaging has not yet been updated.</t>
-  </si>
-  <si>
-    <t>Apply the figures and qualification verbatim, then route external copy through Legal.</t>
+    <t>Mike supplied the approved product specifications; Agent Messaging has not yet been updated.</t>
+  </si>
+  <si>
+    <t>Apply the approved specifications, retaining “up to” and FP4, then route external copy through Legal.</t>
   </si>
   <si>
     <t>DOC_URL</t>
@@ -234,10 +234,10 @@
     <t>Daniel Cho</t>
   </si>
   <si>
-    <t>Daniel cleared Mike’s wording and pre-production qualification for leadership review only.</t>
-  </si>
-  <si>
-    <t>Preserve the qualification and route final external campaign copy through Legal for campaign-wide clearance.</t>
+    <t>Daniel cleared Mike’s product specification wording for leadership review only.</t>
+  </si>
+  <si>
+    <t>Keep “up to” and FP4 intact and route final external campaign copy through Legal for campaign-wide clearance.</t>
   </si>
   <si>
     <t>Campaign-wide clearance remains pending.</t>

</xml_diff>